<commit_message>
Add Evergreen and Loveknot pendants
</commit_message>
<xml_diff>
--- a/business/inventory-ledger.xlsx
+++ b/business/inventory-ledger.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A2AB4CB-51E2-4FB5-8E49-ADB13FC5C6B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0653A177-C768-4A00-AEB6-BDC52C33FCDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{68BF2D20-07EA-4E2C-B5AF-3720521CC247}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{68BF2D20-07EA-4E2C-B5AF-3720521CC247}"/>
   </bookViews>
   <sheets>
     <sheet name="inventory-ledger" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="107">
   <si>
     <t>Product ID</t>
   </si>
@@ -316,6 +316,45 @@
   </si>
   <si>
     <t>10 × 8 × 5</t>
+  </si>
+  <si>
+    <t>Dove</t>
+  </si>
+  <si>
+    <t>JBG-ATN-007</t>
+  </si>
+  <si>
+    <t>Trinity</t>
+  </si>
+  <si>
+    <t>Halo</t>
+  </si>
+  <si>
+    <t>AT-Pendant Set</t>
+  </si>
+  <si>
+    <t>JBG-ATPS-001</t>
+  </si>
+  <si>
+    <t>JBG-ATPS-002</t>
+  </si>
+  <si>
+    <t>Sundrop</t>
+  </si>
+  <si>
+    <t>JBG-ATE-004</t>
+  </si>
+  <si>
+    <t>Evergreen</t>
+  </si>
+  <si>
+    <t>JBG-ATPS-003</t>
+  </si>
+  <si>
+    <t>Loveknot</t>
+  </si>
+  <si>
+    <t>JBG-ATPS-004</t>
   </si>
 </sst>
 </file>
@@ -1836,7 +1875,7 @@
     </row>
     <row r="14" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="str">
-        <f t="shared" ref="A14:A23" si="5">LEFT(A13,4)&amp;TEXT(RIGHT(A13,3)+1,"000")</f>
+        <f t="shared" ref="A14:A29" si="5">LEFT(A13,4)&amp;TEXT(RIGHT(A13,3)+1,"000")</f>
         <v>JBG-013</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -2245,21 +2284,21 @@
         <v>150</v>
       </c>
       <c r="H22" s="1">
-        <f t="shared" ref="H22:H23" si="20">SUM(E22:G22)</f>
+        <f t="shared" ref="H22:H24" si="20">SUM(E22:G22)</f>
         <v>360</v>
       </c>
       <c r="I22" s="1">
         <v>3</v>
       </c>
       <c r="J22" s="1">
-        <f t="shared" ref="J22:J23" si="21">ROUNDUP((H22*I22)/500,0)*500-1</f>
+        <f t="shared" ref="J22:J26" si="21">ROUNDUP((H22*I22)/500,0)*500-1</f>
         <v>1499</v>
       </c>
       <c r="K22" s="1">
         <v>2</v>
       </c>
       <c r="M22" s="1">
-        <f t="shared" ref="M22:M23" si="22">K22-L22</f>
+        <f t="shared" ref="M22:M26" si="22">K22-L22</f>
         <v>2</v>
       </c>
       <c r="N22" s="1" t="s">
@@ -2317,12 +2356,294 @@
         <v>81</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="25" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="26" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="27" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="28" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="24" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>JBG-023</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="1">
+        <v>450</v>
+      </c>
+      <c r="F24" s="1">
+        <v>50</v>
+      </c>
+      <c r="G24" s="1">
+        <v>150</v>
+      </c>
+      <c r="H24" s="1">
+        <f t="shared" si="20"/>
+        <v>650</v>
+      </c>
+      <c r="I24" s="1">
+        <v>2</v>
+      </c>
+      <c r="J24" s="1">
+        <f t="shared" si="21"/>
+        <v>1499</v>
+      </c>
+      <c r="K24" s="1">
+        <v>3</v>
+      </c>
+      <c r="M24" s="1">
+        <f t="shared" si="22"/>
+        <v>3</v>
+      </c>
+      <c r="N24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>JBG-024</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" s="1">
+        <v>130</v>
+      </c>
+      <c r="F25" s="1">
+        <v>50</v>
+      </c>
+      <c r="G25" s="1">
+        <v>150</v>
+      </c>
+      <c r="H25" s="1">
+        <f t="shared" ref="H25:H26" si="23">SUM(E25:G25)</f>
+        <v>330</v>
+      </c>
+      <c r="I25" s="1">
+        <v>2</v>
+      </c>
+      <c r="J25" s="1">
+        <f t="shared" si="21"/>
+        <v>999</v>
+      </c>
+      <c r="K25" s="1">
+        <v>2</v>
+      </c>
+      <c r="M25" s="1">
+        <f t="shared" si="22"/>
+        <v>2</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>JBG-025</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E26" s="1">
+        <v>145</v>
+      </c>
+      <c r="F26" s="1">
+        <v>50</v>
+      </c>
+      <c r="G26" s="1">
+        <v>150</v>
+      </c>
+      <c r="H26" s="1">
+        <f t="shared" si="23"/>
+        <v>345</v>
+      </c>
+      <c r="I26" s="1">
+        <v>2</v>
+      </c>
+      <c r="J26" s="1">
+        <f t="shared" si="21"/>
+        <v>999</v>
+      </c>
+      <c r="K26" s="1">
+        <v>2</v>
+      </c>
+      <c r="M26" s="1">
+        <f t="shared" si="22"/>
+        <v>2</v>
+      </c>
+      <c r="N26" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>JBG-026</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E27" s="1">
+        <v>480</v>
+      </c>
+      <c r="F27" s="1">
+        <v>50</v>
+      </c>
+      <c r="G27" s="1">
+        <v>150</v>
+      </c>
+      <c r="H27" s="1">
+        <f t="shared" ref="H27:H28" si="24">SUM(E27:G27)</f>
+        <v>680</v>
+      </c>
+      <c r="I27" s="1">
+        <v>2</v>
+      </c>
+      <c r="J27" s="1">
+        <f t="shared" ref="J27:J28" si="25">ROUNDUP((H27*I27)/500,0)*500-1</f>
+        <v>1499</v>
+      </c>
+      <c r="K27" s="1">
+        <v>2</v>
+      </c>
+      <c r="M27" s="1">
+        <f t="shared" ref="M27:M28" si="26">K27-L27</f>
+        <v>2</v>
+      </c>
+      <c r="N27" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O27" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>JBG-027</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E28" s="1">
+        <v>149</v>
+      </c>
+      <c r="F28" s="1">
+        <v>50</v>
+      </c>
+      <c r="G28" s="1">
+        <v>150</v>
+      </c>
+      <c r="H28" s="1">
+        <f t="shared" si="24"/>
+        <v>349</v>
+      </c>
+      <c r="I28" s="1">
+        <v>2</v>
+      </c>
+      <c r="J28" s="1">
+        <f t="shared" si="25"/>
+        <v>999</v>
+      </c>
+      <c r="K28" s="1">
+        <v>2</v>
+      </c>
+      <c r="M28" s="1">
+        <f t="shared" si="26"/>
+        <v>2</v>
+      </c>
+      <c r="N28" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O28" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>JBG-028</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E29" s="1">
+        <v>99</v>
+      </c>
+      <c r="F29" s="1">
+        <v>50</v>
+      </c>
+      <c r="G29" s="1">
+        <v>150</v>
+      </c>
+      <c r="H29" s="1">
+        <f t="shared" ref="H29" si="27">SUM(E29:G29)</f>
+        <v>299</v>
+      </c>
+      <c r="I29" s="1">
+        <v>2</v>
+      </c>
+      <c r="J29" s="1">
+        <f t="shared" ref="J29" si="28">ROUNDUP((H29*I29)/500,0)*500-1</f>
+        <v>999</v>
+      </c>
+      <c r="K29" s="1">
+        <v>2</v>
+      </c>
+      <c r="M29" s="1">
+        <f t="shared" ref="M29" si="29">K29-L29</f>
+        <v>2</v>
+      </c>
+      <c r="N29" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O29" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
     <row r="30" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="31" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>